<commit_message>
[wip] attack pipline 5
</commit_message>
<xml_diff>
--- a/table_config/_tables/enums__.xlsx
+++ b/table_config/_tables/enums__.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25420" windowHeight="7120"/>
+    <workbookView windowWidth="25420" windowHeight="7720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>##var</t>
   </si>
@@ -84,6 +84,30 @@
   </si>
   <si>
     <t>注释</t>
+  </si>
+  <si>
+    <t>Battle.Attribute</t>
+  </si>
+  <si>
+    <t>health</t>
+  </si>
+  <si>
+    <t>生命</t>
+  </si>
+  <si>
+    <t>attack</t>
+  </si>
+  <si>
+    <t>攻击</t>
+  </si>
+  <si>
+    <t>Battle.Tag</t>
+  </si>
+  <si>
+    <t>nondamageable</t>
+  </si>
+  <si>
+    <t>免疫伤害</t>
   </si>
   <si>
     <t>Battle.DamageSource</t>
@@ -1109,7 +1133,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="6.45454545454545" customWidth="1"/>
@@ -1120,9 +1144,9 @@
     <col min="6" max="6" width="11.8181818181818" customWidth="1"/>
     <col min="7" max="7" width="5.18181818181818" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="26.6363636363636" customWidth="1"/>
+    <col min="9" max="9" width="15.5454545454545" customWidth="1"/>
     <col min="10" max="10" width="8" style="1" customWidth="1"/>
-    <col min="11" max="11" width="47" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="5.18181818181818" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1213,6 +1237,7 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" spans="1:12">
+      <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
@@ -1232,11 +1257,12 @@
       </c>
       <c r="K4" s="5" t="str">
         <f>I4</f>
-        <v>主要伤害</v>
+        <v>生命</v>
       </c>
       <c r="L4" s="5"/>
     </row>
     <row r="5" spans="1:12">
+      <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -1254,88 +1280,84 @@
       </c>
       <c r="K5" s="5" t="str">
         <f>I5</f>
-        <v>派生伤害</v>
+        <v>攻击</v>
       </c>
       <c r="L5" s="5"/>
     </row>
     <row r="6" spans="1:12">
+      <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" s="6">
-        <v>3</v>
-      </c>
-      <c r="K6" s="5" t="str">
-        <f>I6</f>
-        <v>反弹伤害</v>
-      </c>
-      <c r="L6" s="5"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="5"/>
+      <c r="H7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="6">
+        <v>1</v>
+      </c>
+      <c r="K7" s="5" t="str">
+        <f>I7</f>
+        <v>免疫伤害</v>
+      </c>
       <c r="L7" s="5"/>
     </row>
     <row r="8" spans="1:12">
-      <c r="B8" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="J8" s="6">
-        <v>1</v>
-      </c>
-      <c r="K8" s="5" t="str">
-        <f>I8</f>
-        <v>物理伤害</v>
-      </c>
-      <c r="L8" s="5"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" s="6">
-        <v>2</v>
+      <c r="J9" s="7">
+        <v>1</v>
       </c>
       <c r="K9" s="5" t="str">
         <f>I9</f>
-        <v>魔法伤害</v>
+        <v>主要伤害</v>
       </c>
       <c r="L9" s="5"/>
     </row>
@@ -1346,16 +1368,23 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="5"/>
+      <c r="H10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J10" s="7">
+        <v>2</v>
+      </c>
+      <c r="K10" s="5" t="str">
+        <f>I10</f>
+        <v>派生伤害</v>
+      </c>
       <c r="L10" s="5"/>
     </row>
     <row r="11" spans="1:12">
-      <c r="B11" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -1367,12 +1396,12 @@
       <c r="I11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J11" s="6">
-        <v>1</v>
+      <c r="J11" s="7">
+        <v>3</v>
       </c>
       <c r="K11" s="5" t="str">
         <f>I11</f>
-        <v>基础毒伤害</v>
+        <v>反弹伤害</v>
       </c>
       <c r="L11" s="5"/>
     </row>
@@ -1385,21 +1414,32 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="6"/>
+      <c r="J12" s="7"/>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="B13" s="5"/>
+      <c r="B13" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J13" s="7">
+        <v>1</v>
+      </c>
+      <c r="K13" s="5" t="str">
+        <f>I13</f>
+        <v>物理伤害</v>
+      </c>
       <c r="L13" s="5"/>
     </row>
     <row r="14" spans="1:12">
@@ -1409,10 +1449,19 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="5"/>
+      <c r="H14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J14" s="7">
+        <v>2</v>
+      </c>
+      <c r="K14" s="5" t="str">
+        <f>I14</f>
+        <v>魔法伤害</v>
+      </c>
       <c r="L14" s="5"/>
     </row>
     <row r="15" spans="1:12">
@@ -1424,21 +1473,32 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="5"/>
       <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:12">
-      <c r="B16" s="5"/>
+      <c r="B16" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="5"/>
+      <c r="H16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J16" s="7">
+        <v>1</v>
+      </c>
+      <c r="K16" s="5" t="str">
+        <f>I16</f>
+        <v>基础毒伤害</v>
+      </c>
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:12">
@@ -1450,7 +1510,7 @@
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
-      <c r="J17" s="6"/>
+      <c r="J17" s="7"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
     </row>
@@ -1463,7 +1523,7 @@
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
-      <c r="J18" s="6"/>
+      <c r="J18" s="7"/>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
     </row>
@@ -1476,7 +1536,7 @@
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
-      <c r="J19" s="6"/>
+      <c r="J19" s="7"/>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
     </row>
@@ -1489,8 +1549,8 @@
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="5"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
       <c r="L20" s="5"/>
     </row>
     <row r="21" spans="1:12">
@@ -1502,12 +1562,11 @@
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="6"/>
+      <c r="J21" s="7"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
     </row>
     <row r="22" spans="1:12">
-      <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -1516,12 +1575,11 @@
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="7"/>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
     </row>
     <row r="23" spans="1:12">
-      <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -1530,7 +1588,7 @@
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
-      <c r="J23" s="6"/>
+      <c r="J23" s="7"/>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
     </row>
@@ -1543,7 +1601,7 @@
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="7"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
     </row>
@@ -1556,7 +1614,7 @@
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="7"/>
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
     </row>
@@ -1569,11 +1627,12 @@
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
-      <c r="J26" s="6"/>
+      <c r="J26" s="7"/>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
     </row>
     <row r="27" spans="1:12">
+      <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -1582,11 +1641,12 @@
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="7"/>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
     </row>
     <row r="28" spans="1:12">
+      <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -1595,7 +1655,7 @@
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="7"/>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
     </row>
@@ -1608,7 +1668,7 @@
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
-      <c r="J29" s="6"/>
+      <c r="J29" s="7"/>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
     </row>
@@ -1621,7 +1681,7 @@
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="7"/>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
     </row>
@@ -1634,7 +1694,7 @@
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="7"/>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
     </row>
@@ -1647,7 +1707,7 @@
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
-      <c r="J32" s="6"/>
+      <c r="J32" s="7"/>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
     </row>
@@ -1660,7 +1720,7 @@
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
-      <c r="J33" s="6"/>
+      <c r="J33" s="7"/>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
     </row>
@@ -1673,7 +1733,7 @@
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
-      <c r="J34" s="6"/>
+      <c r="J34" s="7"/>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
     </row>
@@ -1686,7 +1746,7 @@
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
-      <c r="J35" s="6"/>
+      <c r="J35" s="7"/>
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
     </row>
@@ -1699,7 +1759,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
-      <c r="J36" s="6"/>
+      <c r="J36" s="7"/>
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
     </row>
@@ -1712,7 +1772,7 @@
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
-      <c r="J37" s="6"/>
+      <c r="J37" s="7"/>
       <c r="K37" s="5"/>
       <c r="L37" s="5"/>
     </row>
@@ -1725,7 +1785,7 @@
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="7"/>
       <c r="K38" s="5"/>
       <c r="L38" s="5"/>
     </row>
@@ -1738,7 +1798,7 @@
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
-      <c r="J39" s="6"/>
+      <c r="J39" s="7"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
     </row>
@@ -1751,7 +1811,7 @@
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="7"/>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
     </row>
@@ -1764,7 +1824,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
-      <c r="J41" s="6"/>
+      <c r="J41" s="7"/>
       <c r="K41" s="5"/>
       <c r="L41" s="5"/>
     </row>
@@ -1777,7 +1837,7 @@
       <c r="G42" s="5"/>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
-      <c r="J42" s="6"/>
+      <c r="J42" s="7"/>
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
     </row>
@@ -1790,7 +1850,7 @@
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
-      <c r="J43" s="6"/>
+      <c r="J43" s="7"/>
       <c r="K43" s="5"/>
       <c r="L43" s="5"/>
     </row>
@@ -1803,7 +1863,7 @@
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="7"/>
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
     </row>
@@ -1816,7 +1876,7 @@
       <c r="G45" s="5"/>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="7"/>
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
     </row>
@@ -1829,7 +1889,7 @@
       <c r="G46" s="5"/>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
-      <c r="J46" s="6"/>
+      <c r="J46" s="7"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
     </row>
@@ -1842,7 +1902,7 @@
       <c r="G47" s="5"/>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
-      <c r="J47" s="6"/>
+      <c r="J47" s="7"/>
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
     </row>
@@ -1855,7 +1915,7 @@
       <c r="G48" s="5"/>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="7"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
     </row>
@@ -1868,7 +1928,7 @@
       <c r="G49" s="5"/>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="7"/>
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
     </row>
@@ -1881,7 +1941,7 @@
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="7"/>
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
     </row>
@@ -1894,7 +1954,7 @@
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="7"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
     </row>
@@ -1907,7 +1967,7 @@
       <c r="G52" s="5"/>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="7"/>
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
     </row>
@@ -1920,7 +1980,7 @@
       <c r="G53" s="5"/>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="7"/>
       <c r="K53" s="5"/>
       <c r="L53" s="5"/>
     </row>
@@ -1933,7 +1993,7 @@
       <c r="G54" s="5"/>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="7"/>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
     </row>
@@ -1946,7 +2006,7 @@
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="7"/>
       <c r="K55" s="5"/>
       <c r="L55" s="5"/>
     </row>
@@ -1959,7 +2019,7 @@
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
       <c r="I56" s="5"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="7"/>
       <c r="K56" s="5"/>
       <c r="L56" s="5"/>
     </row>
@@ -1972,7 +2032,7 @@
       <c r="G57" s="5"/>
       <c r="H57" s="5"/>
       <c r="I57" s="5"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="7"/>
       <c r="K57" s="5"/>
       <c r="L57" s="5"/>
     </row>
@@ -1985,7 +2045,7 @@
       <c r="G58" s="5"/>
       <c r="H58" s="5"/>
       <c r="I58" s="5"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="7"/>
       <c r="K58" s="5"/>
       <c r="L58" s="5"/>
     </row>
@@ -1998,7 +2058,7 @@
       <c r="G59" s="5"/>
       <c r="H59" s="5"/>
       <c r="I59" s="5"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="7"/>
       <c r="K59" s="5"/>
       <c r="L59" s="5"/>
     </row>
@@ -2011,7 +2071,7 @@
       <c r="G60" s="5"/>
       <c r="H60" s="5"/>
       <c r="I60" s="5"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="7"/>
       <c r="K60" s="5"/>
       <c r="L60" s="5"/>
     </row>
@@ -2024,7 +2084,7 @@
       <c r="G61" s="5"/>
       <c r="H61" s="5"/>
       <c r="I61" s="5"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="7"/>
       <c r="K61" s="5"/>
       <c r="L61" s="5"/>
     </row>
@@ -2037,7 +2097,7 @@
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
       <c r="I62" s="5"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="7"/>
       <c r="K62" s="5"/>
       <c r="L62" s="5"/>
     </row>
@@ -2050,7 +2110,7 @@
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
       <c r="I63" s="5"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="7"/>
       <c r="K63" s="5"/>
       <c r="L63" s="5"/>
     </row>
@@ -2063,7 +2123,7 @@
       <c r="G64" s="5"/>
       <c r="H64" s="5"/>
       <c r="I64" s="5"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="7"/>
       <c r="K64" s="5"/>
       <c r="L64" s="5"/>
     </row>
@@ -2076,7 +2136,7 @@
       <c r="G65" s="5"/>
       <c r="H65" s="5"/>
       <c r="I65" s="5"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="7"/>
       <c r="K65" s="5"/>
       <c r="L65" s="5"/>
     </row>
@@ -2089,7 +2149,7 @@
       <c r="G66" s="5"/>
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="7"/>
       <c r="K66" s="5"/>
       <c r="L66" s="5"/>
     </row>
@@ -2102,7 +2162,7 @@
       <c r="G67" s="5"/>
       <c r="H67" s="5"/>
       <c r="I67" s="5"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="7"/>
       <c r="K67" s="5"/>
       <c r="L67" s="5"/>
     </row>
@@ -2115,7 +2175,7 @@
       <c r="G68" s="5"/>
       <c r="H68" s="5"/>
       <c r="I68" s="5"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="7"/>
       <c r="K68" s="5"/>
       <c r="L68" s="5"/>
     </row>
@@ -2128,7 +2188,7 @@
       <c r="G69" s="5"/>
       <c r="H69" s="5"/>
       <c r="I69" s="5"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="7"/>
       <c r="K69" s="5"/>
       <c r="L69" s="5"/>
     </row>
@@ -2141,7 +2201,7 @@
       <c r="G70" s="5"/>
       <c r="H70" s="5"/>
       <c r="I70" s="5"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="7"/>
       <c r="K70" s="5"/>
       <c r="L70" s="5"/>
     </row>
@@ -2154,7 +2214,7 @@
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
       <c r="I71" s="5"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="7"/>
       <c r="K71" s="5"/>
       <c r="L71" s="5"/>
     </row>
@@ -2167,7 +2227,7 @@
       <c r="G72" s="5"/>
       <c r="H72" s="5"/>
       <c r="I72" s="5"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="7"/>
       <c r="K72" s="5"/>
       <c r="L72" s="5"/>
     </row>
@@ -2180,7 +2240,7 @@
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
       <c r="I73" s="5"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="7"/>
       <c r="K73" s="5"/>
       <c r="L73" s="5"/>
     </row>
@@ -2193,7 +2253,7 @@
       <c r="G74" s="5"/>
       <c r="H74" s="5"/>
       <c r="I74" s="5"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="7"/>
       <c r="K74" s="5"/>
       <c r="L74" s="5"/>
     </row>
@@ -2206,7 +2266,7 @@
       <c r="G75" s="5"/>
       <c r="H75" s="5"/>
       <c r="I75" s="5"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="7"/>
       <c r="K75" s="5"/>
       <c r="L75" s="5"/>
     </row>
@@ -2219,7 +2279,7 @@
       <c r="G76" s="5"/>
       <c r="H76" s="5"/>
       <c r="I76" s="5"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="7"/>
       <c r="K76" s="5"/>
       <c r="L76" s="5"/>
     </row>
@@ -2232,7 +2292,7 @@
       <c r="G77" s="5"/>
       <c r="H77" s="5"/>
       <c r="I77" s="5"/>
-      <c r="J77" s="6"/>
+      <c r="J77" s="7"/>
       <c r="K77" s="5"/>
       <c r="L77" s="5"/>
     </row>
@@ -2245,7 +2305,7 @@
       <c r="G78" s="5"/>
       <c r="H78" s="5"/>
       <c r="I78" s="5"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="7"/>
       <c r="K78" s="5"/>
       <c r="L78" s="5"/>
     </row>
@@ -2258,7 +2318,7 @@
       <c r="G79" s="5"/>
       <c r="H79" s="5"/>
       <c r="I79" s="5"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="7"/>
       <c r="K79" s="5"/>
       <c r="L79" s="5"/>
     </row>
@@ -2271,7 +2331,7 @@
       <c r="G80" s="5"/>
       <c r="H80" s="5"/>
       <c r="I80" s="5"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="7"/>
       <c r="K80" s="5"/>
       <c r="L80" s="5"/>
     </row>
@@ -2284,7 +2344,7 @@
       <c r="G81" s="5"/>
       <c r="H81" s="5"/>
       <c r="I81" s="5"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="7"/>
       <c r="K81" s="5"/>
       <c r="L81" s="5"/>
     </row>
@@ -2297,7 +2357,7 @@
       <c r="G82" s="5"/>
       <c r="H82" s="5"/>
       <c r="I82" s="5"/>
-      <c r="J82" s="6"/>
+      <c r="J82" s="7"/>
       <c r="K82" s="5"/>
       <c r="L82" s="5"/>
     </row>
@@ -2310,7 +2370,7 @@
       <c r="G83" s="5"/>
       <c r="H83" s="5"/>
       <c r="I83" s="5"/>
-      <c r="J83" s="6"/>
+      <c r="J83" s="7"/>
       <c r="K83" s="5"/>
       <c r="L83" s="5"/>
     </row>
@@ -2323,7 +2383,7 @@
       <c r="G84" s="5"/>
       <c r="H84" s="5"/>
       <c r="I84" s="5"/>
-      <c r="J84" s="6"/>
+      <c r="J84" s="7"/>
       <c r="K84" s="5"/>
       <c r="L84" s="5"/>
     </row>
@@ -2336,7 +2396,7 @@
       <c r="G85" s="5"/>
       <c r="H85" s="5"/>
       <c r="I85" s="5"/>
-      <c r="J85" s="6"/>
+      <c r="J85" s="7"/>
       <c r="K85" s="5"/>
       <c r="L85" s="5"/>
     </row>
@@ -2349,7 +2409,7 @@
       <c r="G86" s="5"/>
       <c r="H86" s="5"/>
       <c r="I86" s="5"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="7"/>
       <c r="K86" s="5"/>
       <c r="L86" s="5"/>
     </row>
@@ -2362,7 +2422,7 @@
       <c r="G87" s="5"/>
       <c r="H87" s="5"/>
       <c r="I87" s="5"/>
-      <c r="J87" s="6"/>
+      <c r="J87" s="7"/>
       <c r="K87" s="5"/>
       <c r="L87" s="5"/>
     </row>
@@ -2375,7 +2435,7 @@
       <c r="G88" s="5"/>
       <c r="H88" s="5"/>
       <c r="I88" s="5"/>
-      <c r="J88" s="6"/>
+      <c r="J88" s="7"/>
       <c r="K88" s="5"/>
       <c r="L88" s="5"/>
     </row>
@@ -2388,9 +2448,74 @@
       <c r="G89" s="5"/>
       <c r="H89" s="5"/>
       <c r="I89" s="5"/>
-      <c r="J89" s="6"/>
+      <c r="J89" s="7"/>
       <c r="K89" s="5"/>
       <c r="L89" s="5"/>
+    </row>
+    <row r="90" spans="2:12">
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="7"/>
+      <c r="K90" s="5"/>
+      <c r="L90" s="5"/>
+    </row>
+    <row r="91" spans="2:12">
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="7"/>
+      <c r="K91" s="5"/>
+      <c r="L91" s="5"/>
+    </row>
+    <row r="92" spans="2:12">
+      <c r="B92" s="5"/>
+      <c r="C92" s="5"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
+      <c r="I92" s="5"/>
+      <c r="J92" s="7"/>
+      <c r="K92" s="5"/>
+      <c r="L92" s="5"/>
+    </row>
+    <row r="93" spans="2:12">
+      <c r="B93" s="5"/>
+      <c r="C93" s="5"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5"/>
+      <c r="I93" s="5"/>
+      <c r="J93" s="7"/>
+      <c r="K93" s="5"/>
+      <c r="L93" s="5"/>
+    </row>
+    <row r="94" spans="2:12">
+      <c r="B94" s="5"/>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="5"/>
+      <c r="J94" s="7"/>
+      <c r="K94" s="5"/>
+      <c r="L94" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>